<commit_message>
Fix: Remove duplicate SO-306 row causing scheduler NaN error
Root cause analysis identified that row 312 in Sales_Orders sheet contained a duplicate SO-306 entry with a different SKU. This created conflicting campaign data and caused the scheduler to receive NaN values when computing due dates.

Changes:
- Deleted row 312 (duplicate SO-306 entry) from Sales_Orders sheet in APS_BF_SMS_RM.xlsx
- Also updated data validation filters in _load_all() to remove SO_ID='nan' string entries (header/description rows)
- Changed datetime parsing to use format='mixed' to handle mixed date formats properly

Result: API /run/schedule endpoint now works correctly without NaN errors. Scheduler returns valid results.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APS_BF_SMS_RM.xlsx
+++ b/APS_BF_SMS_RM.xlsx
@@ -29740,7 +29740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N313"/>
+  <dimension ref="A1:N311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" style="39" min="1" max="1"/>
@@ -48892,111 +48892,6 @@
         <is>
           <t>Backlog</t>
         </is>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" t="inlineStr">
-        <is>
-          <t>SO-306</t>
-        </is>
-      </c>
-      <c r="B312" t="inlineStr">
-        <is>
-          <t>Kalyani Carpenter</t>
-        </is>
-      </c>
-      <c r="C312" t="inlineStr">
-        <is>
-          <t>South</t>
-        </is>
-      </c>
-      <c r="D312" t="inlineStr">
-        <is>
-          <t>FG-WR-CHQ1006-55</t>
-        </is>
-      </c>
-      <c r="E312" t="inlineStr">
-        <is>
-          <t>CHQ 1006</t>
-        </is>
-      </c>
-      <c r="F312" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="G312" t="n">
-        <v>60</v>
-      </c>
-      <c r="H312" t="n">
-        <v>30</v>
-      </c>
-      <c r="I312" s="48" t="n">
-        <v>46116</v>
-      </c>
-      <c r="J312" s="48" t="n">
-        <v>46122</v>
-      </c>
-      <c r="K312" t="inlineStr">
-        <is>
-          <t>URGENT</t>
-        </is>
-      </c>
-      <c r="L312" t="inlineStr">
-        <is>
-          <t>CHQ-RUSH</t>
-        </is>
-      </c>
-      <c r="N312" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="313">
-      <c r="A313" t="inlineStr">
-        <is>
-          <t>SO-306</t>
-        </is>
-      </c>
-      <c r="B313" t="inlineStr">
-        <is>
-          <t>Kalyani Carpenter</t>
-        </is>
-      </c>
-      <c r="C313" t="inlineStr">
-        <is>
-          <t>FG-WR-CHQ1006-55</t>
-        </is>
-      </c>
-      <c r="D313" t="inlineStr">
-        <is>
-          <t>CHQ 1006</t>
-        </is>
-      </c>
-      <c r="E313" t="inlineStr">
-        <is>
-          <t>5.5mm</t>
-        </is>
-      </c>
-      <c r="F313" t="n">
-        <v>60</v>
-      </c>
-      <c r="G313" t="inlineStr">
-        <is>
-          <t>2026-04-10</t>
-        </is>
-      </c>
-      <c r="H313" t="inlineStr">
-        <is>
-          <t>URGENT</t>
-        </is>
-      </c>
-      <c r="I313" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="J313" s="51" t="n">
-        <v>46122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix: Filter out null SO_ID rows in Sales Orders tab rendering
The Sales_Orders sheet contains empty rows (with null SO_ID) mixed in with valid orders. The API was returning these empty rows, causing the UI to display empty order cards with dashes.

Fixed by adding a client-side filter in renderOrders() to exclude orders where SO_ID is null or empty. This ensures only valid sales orders are displayed in the table.

Changes:
- ui_design/index.html: Added SO_ID validation check in renderOrders()
- ui_design/xaps_iframe_app.html: Added SO_ID validation check in renderOrders()
- xaps_application_api.py: Added SO_ID filter in aps_orders_list() endpoint

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APS_BF_SMS_RM.xlsx
+++ b/APS_BF_SMS_RM.xlsx
@@ -8217,7 +8217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" customWidth="1" style="39" min="1" max="4"/>
@@ -8467,6 +8467,86 @@
       <c r="D12" t="inlineStr">
         <is>
           <t>2026-04-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>REQ-1775322199163</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>FG-WR-SAE1080-55</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>120</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>REQ-1775322214774</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>FG-WR-SAE1080-55</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>120</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>REQ-1775322228329</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>FG-WR-SAE1008-55</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>120</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>REQ-1775452162143</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>FG-WR-SAE1008-65</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Checkpoint: Campaign-based planning page (incorrect foundation)
Work-in-progress state before architectural rebuild.

Added:
- engine/rolling_campaign.py (PO generator, not to be used)
- Planning page with 3-panel UI (will be replaced)
- API endpoints for campaign-based planning
- Design documentation (APS Design Philosophy, ROLLING_CAMPAIGN_MODEL, UI_PLANNING_WORKFLOW)

These are based on incorrect campaign-first architecture and will be
superseded by SO → Planning Order → Heat → Schedule model.

Status: Committing as checkpoint before complete redesign per APS Design Philosophy.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APS_BF_SMS_RM.xlsx
+++ b/APS_BF_SMS_RM.xlsx
@@ -3699,7 +3699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P51"/>
+  <dimension ref="A1:P76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="26" customWidth="1" style="39" min="1" max="1"/>
@@ -4677,7 +4677,7 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>RM-01</t>
+          <t>RM-02</t>
         </is>
       </c>
       <c r="H17" s="4" t="n">
@@ -4741,7 +4741,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>RM-01</t>
+          <t>RM-02</t>
         </is>
       </c>
       <c r="H18" s="4" t="n">
@@ -4805,7 +4805,7 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>RM-01</t>
+          <t>RM-02</t>
         </is>
       </c>
       <c r="H19" s="4" t="n">
@@ -4869,7 +4869,7 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>RM-01</t>
+          <t>RM-02</t>
         </is>
       </c>
       <c r="H20" s="4" t="n">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>RM-01</t>
+          <t>RM-02</t>
         </is>
       </c>
       <c r="H21" s="4" t="n">
@@ -4997,7 +4997,7 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>RM-01</t>
+          <t>RM-02</t>
         </is>
       </c>
       <c r="H22" s="4" t="n">
@@ -5061,7 +5061,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>RM-01</t>
+          <t>RM-02</t>
         </is>
       </c>
       <c r="H23" s="4" t="n">
@@ -5125,7 +5125,7 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>RM-01</t>
+          <t>RM-02</t>
         </is>
       </c>
       <c r="H24" s="4" t="n">
@@ -6605,7 +6605,7 @@
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>CCM-01</t>
+          <t>CCM-02</t>
         </is>
       </c>
       <c r="H47" s="4" t="n">
@@ -6896,6 +6896,431 @@
       <c r="O51" s="4" t="n"/>
       <c r="P51" s="4" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1008-55</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>RM-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1008-65</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>RM-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1008-80</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>RM-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1018-55</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>RM-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1018-65</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>RM-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1018-80</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>RM-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1018-100</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>RM-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1018-120</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>RM-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1035-65</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>RM-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1035-80</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>RM-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1045-65</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>RM-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1045-80</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>RM-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1045-100</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>RM-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1065-55</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>RM-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1065-65</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>RM-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1080-55</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>RM-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>RM-OUT-SAE1080-65</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>RM-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>RM-OUT-CHQ1006-55</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>RM-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>RM-OUT-CHQ1006-65</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>RM-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>RM-OUT-CrMo4140-80</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>RM-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>RM-OUT-CrMo4140-100</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>RM-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>VD-OUT-SAE1065</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Degassing</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>VD-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>VD-OUT-SAE1080</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Degassing</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>VD-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>VD-OUT-CHQ1006</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Degassing</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>VD-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>VD-OUT-CrMo4140</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Degassing</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>VD-01</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -8217,7 +8642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" customWidth="1" style="39" min="1" max="4"/>
@@ -8545,6 +8970,26 @@
         <v>1</v>
       </c>
       <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>REQ-1775465786479</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>FG-WR-SAE1008-80</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>12</v>
+      </c>
+      <c r="D17" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
@@ -30007,7 +30452,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>CMP-003</t>
+          <t>CMP-002</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
@@ -30247,7 +30692,11 @@
           <t>CMP-SAE101</t>
         </is>
       </c>
-      <c r="M10" s="11" t="n"/>
+      <c r="M10" s="11" t="inlineStr">
+        <is>
+          <t>CMP-005</t>
+        </is>
+      </c>
       <c r="N10" s="11" t="inlineStr">
         <is>
           <t>Open</t>
@@ -30311,7 +30760,7 @@
       </c>
       <c r="M11" s="10" t="inlineStr">
         <is>
-          <t>CMP-003</t>
+          <t>CMP-007</t>
         </is>
       </c>
       <c r="N11" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Feat: Integrate BOM explosion into Planning workflow with material constraint analysis
- Promote BOM tab next to Planning tab for visibility
- Add SKU/Material columns to SO, PO, and Heat tables
- Implement [Material] button to check material requirements per SO/PO
- Add material side panel showing BOM tree and inventory status
- Reuse existing BOM rendering logic for consistency
- Store gross_bom data in state for material checks
- Show material status indicators (COVERED/PARTIAL/SHORT)

This enables planners to review material constraints during PO creation.
</commit_message>
<xml_diff>
--- a/APS_BF_SMS_RM.xlsx
+++ b/APS_BF_SMS_RM.xlsx
@@ -8549,7 +8549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" customWidth="1" style="35" min="1" max="4"/>
@@ -8899,6 +8899,23 @@
       <c r="D17" t="inlineStr">
         <is>
           <t>2026-04-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>REQ-1775562304948</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>FG-WR-SAE1008-80</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: implement feasibility filter functionality (priority, resources, horizon)
Backend:
- Read priority_filter, num_sms, num_rm, horizon_hours from simulate request payload
- Apply priority filtering to planning orders before scheduling
- Reduce SMS/RM resource capacity based on num_sms/num_rm parameters
- Convert horizon_hours to planning_horizon_days
- Suppress stdout during scheduler to avoid Windows Unicode encoding errors

Data Model:
- Add priority field to PlanningOrder dataclass
- Compute PO priority as highest (most urgent) from constituent SOs
- Include priority in PlanningOrder.to_dict()

Results:
- Filters now produce measurable impact: narrowing priority window reduces schedule duration
- Example: 30 POs in 377h, URGENT only 9 POs in 124h, URGENT+HIGH 24 POs in 314h
- Remediation controls now actually work instead of being UI theater

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APS_BF_SMS_RM.xlsx
+++ b/APS_BF_SMS_RM.xlsx
@@ -33112,7 +33112,7 @@
       </c>
       <c r="O39" s="11" t="inlineStr">
         <is>
-          <t>PO-0002</t>
+          <t>PO-0001</t>
         </is>
       </c>
       <c r="P39" s="11" t="inlineStr">
@@ -33178,7 +33178,7 @@
       </c>
       <c r="O40" s="11" t="inlineStr">
         <is>
-          <t>PO-0005</t>
+          <t>PO-0002</t>
         </is>
       </c>
       <c r="P40" s="11" t="inlineStr">
@@ -33896,7 +33896,7 @@
       </c>
       <c r="O51" s="11" t="inlineStr">
         <is>
-          <t>PO-0009</t>
+          <t>PO-0003</t>
         </is>
       </c>
       <c r="P51" s="11" t="inlineStr">

</xml_diff>

<commit_message>
chore: update code structure for improved readability and maintainability. Changed the BOM Logic based on which BOM explosion is shown on front end.
</commit_message>
<xml_diff>
--- a/APS_BF_SMS_RM.xlsx
+++ b/APS_BF_SMS_RM.xlsx
@@ -31175,13 +31175,17 @@
       </c>
       <c r="N9" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE103</t>
-        </is>
-      </c>
-      <c r="O9" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>PO-0028</t>
+        </is>
+      </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -32005,13 +32009,17 @@
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE106</t>
-        </is>
-      </c>
-      <c r="O22" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
+        <is>
+          <t>PO-0029</t>
+        </is>
+      </c>
       <c r="P22" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -32199,13 +32207,17 @@
       </c>
       <c r="N25" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE108</t>
-        </is>
-      </c>
-      <c r="O25" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>PO-0030</t>
+        </is>
+      </c>
       <c r="P25" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -32389,13 +32401,17 @@
       </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE100</t>
-        </is>
-      </c>
-      <c r="O28" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O28" s="4" t="inlineStr">
+        <is>
+          <t>PO-0027</t>
+        </is>
+      </c>
       <c r="P28" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -33112,7 +33128,7 @@
       </c>
       <c r="O39" s="11" t="inlineStr">
         <is>
-          <t>PO-0001</t>
+          <t>PO-0002</t>
         </is>
       </c>
       <c r="P39" s="11" t="inlineStr">
@@ -33178,7 +33194,7 @@
       </c>
       <c r="O40" s="11" t="inlineStr">
         <is>
-          <t>PO-0002</t>
+          <t>PO-0005</t>
         </is>
       </c>
       <c r="P40" s="11" t="inlineStr">
@@ -33503,13 +33519,17 @@
       </c>
       <c r="N45" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE103</t>
-        </is>
-      </c>
-      <c r="O45" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
+        <is>
+          <t>PO-0028</t>
+        </is>
+      </c>
       <c r="P45" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -33896,7 +33916,7 @@
       </c>
       <c r="O51" s="11" t="inlineStr">
         <is>
-          <t>PO-0003</t>
+          <t>PO-0009</t>
         </is>
       </c>
       <c r="P51" s="11" t="inlineStr">

</xml_diff>

<commit_message>
chore: consolidate workspace state into main repo
</commit_message>
<xml_diff>
--- a/APS_BF_SMS_RM.xlsx
+++ b/APS_BF_SMS_RM.xlsx
@@ -8549,7 +8549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" customWidth="1" style="35" min="1" max="4"/>
@@ -8916,6 +8916,23 @@
       <c r="D18" t="inlineStr">
         <is>
           <t>2026-04-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>REQ-1775732423862</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>FG-WR-SAE1018-100</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
@@ -30845,17 +30862,17 @@
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE101</t>
+          <t>APS_RELEASED</t>
         </is>
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>CMP-002</t>
+          <t>PO-0025</t>
         </is>
       </c>
       <c r="P4" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -30911,17 +30928,17 @@
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE108</t>
+          <t>APS_RELEASED</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>CMP-001</t>
+          <t>PO-0036</t>
         </is>
       </c>
       <c r="P5" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -31180,7 +31197,7 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>PO-0028</t>
+          <t>PO-0027</t>
         </is>
       </c>
       <c r="P9" s="4" t="inlineStr">
@@ -31757,13 +31774,17 @@
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE103</t>
-        </is>
-      </c>
-      <c r="O18" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>PO-0027</t>
+        </is>
+      </c>
       <c r="P18" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -31947,13 +31968,17 @@
       </c>
       <c r="N21" s="4" t="inlineStr">
         <is>
-          <t>CMP-CrMo41</t>
-        </is>
-      </c>
-      <c r="O21" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>PO-0034</t>
+        </is>
+      </c>
       <c r="P21" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -32014,7 +32039,7 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>PO-0029</t>
+          <t>PO-0032</t>
         </is>
       </c>
       <c r="P22" s="4" t="inlineStr">
@@ -32212,7 +32237,7 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>PO-0030</t>
+          <t>PO-0033</t>
         </is>
       </c>
       <c r="P25" s="4" t="inlineStr">
@@ -32406,7 +32431,7 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>PO-0027</t>
+          <t>PO-0030</t>
         </is>
       </c>
       <c r="P28" s="4" t="inlineStr">
@@ -32533,13 +32558,17 @@
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE101</t>
-        </is>
-      </c>
-      <c r="O30" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O30" s="4" t="inlineStr">
+        <is>
+          <t>PO-0035</t>
+        </is>
+      </c>
       <c r="P30" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -32996,7 +33025,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>PO-0026</t>
+          <t>PO-0029</t>
         </is>
       </c>
       <c r="P37" s="4" t="inlineStr">
@@ -33062,7 +33091,7 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>PO-0025</t>
+          <t>PO-0028</t>
         </is>
       </c>
       <c r="P38" s="4" t="inlineStr">
@@ -33524,7 +33553,7 @@
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>PO-0028</t>
+          <t>PO-0031</t>
         </is>
       </c>
       <c r="P45" s="4" t="inlineStr">
@@ -33585,13 +33614,17 @@
       </c>
       <c r="N46" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE103</t>
-        </is>
-      </c>
-      <c r="O46" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O46" s="4" t="inlineStr">
+        <is>
+          <t>PO-0026</t>
+        </is>
+      </c>
       <c r="P46" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -34695,13 +34728,17 @@
       </c>
       <c r="N63" s="10" t="inlineStr">
         <is>
-          <t>CMP-SAE101</t>
-        </is>
-      </c>
-      <c r="O63" s="10" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O63" s="10" t="inlineStr">
+        <is>
+          <t>PO-0025</t>
+        </is>
+      </c>
       <c r="P63" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -34819,13 +34856,17 @@
       </c>
       <c r="N65" s="10" t="inlineStr">
         <is>
-          <t>CMP-SAE103</t>
-        </is>
-      </c>
-      <c r="O65" s="10" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O65" s="10" t="inlineStr">
+        <is>
+          <t>PO-0026</t>
+        </is>
+      </c>
       <c r="P65" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -34881,13 +34922,17 @@
       </c>
       <c r="N66" s="10" t="inlineStr">
         <is>
-          <t>CMP-SAE103</t>
-        </is>
-      </c>
-      <c r="O66" s="10" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O66" s="10" t="inlineStr">
+        <is>
+          <t>PO-0027</t>
+        </is>
+      </c>
       <c r="P66" s="10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor code structure for improved readability and maintainability. Significant cleanup of styles and consolidation.
</commit_message>
<xml_diff>
--- a/APS_BF_SMS_RM.xlsx
+++ b/APS_BF_SMS_RM.xlsx
@@ -30933,7 +30933,7 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>PO-0036</t>
+          <t>PO-0034</t>
         </is>
       </c>
       <c r="P5" s="4" t="inlineStr">
@@ -30999,7 +30999,7 @@
       </c>
       <c r="O6" s="10" t="inlineStr">
         <is>
-          <t>PO-0009</t>
+          <t>PO-0021</t>
         </is>
       </c>
       <c r="P6" s="10" t="inlineStr">
@@ -31131,7 +31131,7 @@
       </c>
       <c r="O8" s="10" t="inlineStr">
         <is>
-          <t>PO-0018</t>
+          <t>PO-0017</t>
         </is>
       </c>
       <c r="P8" s="10" t="inlineStr">
@@ -31258,13 +31258,17 @@
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE106</t>
-        </is>
-      </c>
-      <c r="O10" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>PO-0038</t>
+        </is>
+      </c>
       <c r="P10" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -31457,7 +31461,7 @@
       </c>
       <c r="O13" s="10" t="inlineStr">
         <is>
-          <t>PO-0014</t>
+          <t>PO-0013</t>
         </is>
       </c>
       <c r="P13" s="10" t="inlineStr">
@@ -31518,13 +31522,17 @@
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE106</t>
-        </is>
-      </c>
-      <c r="O14" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>PO-0030</t>
+        </is>
+      </c>
       <c r="P14" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -31585,7 +31593,7 @@
       </c>
       <c r="O15" s="10" t="inlineStr">
         <is>
-          <t>PO-0013</t>
+          <t>PO-0012</t>
         </is>
       </c>
       <c r="P15" s="10" t="inlineStr">
@@ -31646,13 +31654,17 @@
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE106</t>
-        </is>
-      </c>
-      <c r="O16" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
+          <t>PO-0038</t>
+        </is>
+      </c>
       <c r="P16" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -31840,13 +31852,17 @@
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE101</t>
-        </is>
-      </c>
-      <c r="O19" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>PO-0037</t>
+        </is>
+      </c>
       <c r="P19" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -31973,7 +31989,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>PO-0034</t>
+          <t>PO-0032</t>
         </is>
       </c>
       <c r="P21" s="4" t="inlineStr">
@@ -32039,7 +32055,7 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>PO-0032</t>
+          <t>PO-0030</t>
         </is>
       </c>
       <c r="P22" s="4" t="inlineStr">
@@ -32105,7 +32121,7 @@
       </c>
       <c r="O23" s="10" t="inlineStr">
         <is>
-          <t>PO-0012</t>
+          <t>PO-0011</t>
         </is>
       </c>
       <c r="P23" s="10" t="inlineStr">
@@ -32171,7 +32187,7 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>PO-0021</t>
+          <t>PO-0020</t>
         </is>
       </c>
       <c r="P24" s="4" t="inlineStr">
@@ -32237,7 +32253,7 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>PO-0033</t>
+          <t>PO-0031</t>
         </is>
       </c>
       <c r="P25" s="4" t="inlineStr">
@@ -32298,13 +32314,17 @@
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE101</t>
-        </is>
-      </c>
-      <c r="O26" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>PO-0025</t>
+        </is>
+      </c>
       <c r="P26" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -32431,7 +32451,7 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>PO-0030</t>
+          <t>PO-0021</t>
         </is>
       </c>
       <c r="P28" s="4" t="inlineStr">
@@ -32563,7 +32583,7 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>PO-0035</t>
+          <t>PO-0033</t>
         </is>
       </c>
       <c r="P30" s="4" t="inlineStr">
@@ -32761,7 +32781,7 @@
       </c>
       <c r="O33" s="10" t="inlineStr">
         <is>
-          <t>PO-0010</t>
+          <t>PO-0009</t>
         </is>
       </c>
       <c r="P33" s="10" t="inlineStr">
@@ -32827,7 +32847,7 @@
       </c>
       <c r="O34" s="10" t="inlineStr">
         <is>
-          <t>PO-0011</t>
+          <t>PO-0010</t>
         </is>
       </c>
       <c r="P34" s="10" t="inlineStr">
@@ -32893,7 +32913,7 @@
       </c>
       <c r="O35" s="10" t="inlineStr">
         <is>
-          <t>PO-0015</t>
+          <t>PO-0014</t>
         </is>
       </c>
       <c r="P35" s="10" t="inlineStr">
@@ -32959,7 +32979,7 @@
       </c>
       <c r="O36" s="10" t="inlineStr">
         <is>
-          <t>PO-0019</t>
+          <t>PO-0018</t>
         </is>
       </c>
       <c r="P36" s="10" t="inlineStr">
@@ -33355,7 +33375,7 @@
       </c>
       <c r="O42" s="10" t="inlineStr">
         <is>
-          <t>PO-0020</t>
+          <t>PO-0019</t>
         </is>
       </c>
       <c r="P42" s="10" t="inlineStr">
@@ -33487,7 +33507,7 @@
       </c>
       <c r="O44" s="10" t="inlineStr">
         <is>
-          <t>PO-0018</t>
+          <t>PO-0017</t>
         </is>
       </c>
       <c r="P44" s="10" t="inlineStr">
@@ -33553,7 +33573,7 @@
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>PO-0031</t>
+          <t>PO-0027</t>
         </is>
       </c>
       <c r="P45" s="4" t="inlineStr">
@@ -33680,17 +33700,17 @@
       </c>
       <c r="N47" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE101</t>
+          <t>APS_RELEASED</t>
         </is>
       </c>
       <c r="O47" s="4" t="inlineStr">
         <is>
-          <t>BIG-1018</t>
+          <t>PO-0036</t>
         </is>
       </c>
       <c r="P47" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -33746,17 +33766,17 @@
       </c>
       <c r="N48" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE101</t>
+          <t>APS_RELEASED</t>
         </is>
       </c>
       <c r="O48" s="4" t="inlineStr">
         <is>
-          <t>BIG-1018</t>
+          <t>PO-0036</t>
         </is>
       </c>
       <c r="P48" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -33817,7 +33837,7 @@
       </c>
       <c r="O49" s="10" t="inlineStr">
         <is>
-          <t>PO-0012</t>
+          <t>PO-0011</t>
         </is>
       </c>
       <c r="P49" s="10" t="inlineStr">
@@ -33949,7 +33969,7 @@
       </c>
       <c r="O51" s="11" t="inlineStr">
         <is>
-          <t>PO-0009</t>
+          <t>PO-0002</t>
         </is>
       </c>
       <c r="P51" s="11" t="inlineStr">
@@ -34081,7 +34101,7 @@
       </c>
       <c r="O53" s="10" t="inlineStr">
         <is>
-          <t>PO-0016</t>
+          <t>PO-0015</t>
         </is>
       </c>
       <c r="P53" s="10" t="inlineStr">
@@ -34147,7 +34167,7 @@
       </c>
       <c r="O54" s="10" t="inlineStr">
         <is>
-          <t>PO-0013</t>
+          <t>PO-0012</t>
         </is>
       </c>
       <c r="P54" s="10" t="inlineStr">
@@ -34213,7 +34233,7 @@
       </c>
       <c r="O55" s="10" t="inlineStr">
         <is>
-          <t>PO-0017</t>
+          <t>PO-0016</t>
         </is>
       </c>
       <c r="P55" s="10" t="inlineStr">
@@ -34279,7 +34299,7 @@
       </c>
       <c r="O56" s="10" t="inlineStr">
         <is>
-          <t>PO-0014</t>
+          <t>PO-0013</t>
         </is>
       </c>
       <c r="P56" s="10" t="inlineStr">
@@ -34345,7 +34365,7 @@
       </c>
       <c r="O57" s="10" t="inlineStr">
         <is>
-          <t>PO-0020</t>
+          <t>PO-0019</t>
         </is>
       </c>
       <c r="P57" s="10" t="inlineStr">
@@ -34477,7 +34497,7 @@
       </c>
       <c r="O59" s="10" t="inlineStr">
         <is>
-          <t>PO-0021</t>
+          <t>PO-0020</t>
         </is>
       </c>
       <c r="P59" s="10" t="inlineStr">
@@ -34543,7 +34563,7 @@
       </c>
       <c r="O60" s="10" t="inlineStr">
         <is>
-          <t>PO-0010</t>
+          <t>PO-0009</t>
         </is>
       </c>
       <c r="P60" s="10" t="inlineStr">
@@ -34666,13 +34686,17 @@
       </c>
       <c r="N62" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE100</t>
-        </is>
-      </c>
-      <c r="O62" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O62" s="4" t="inlineStr">
+        <is>
+          <t>PO-0035</t>
+        </is>
+      </c>
       <c r="P62" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -34794,13 +34818,17 @@
       </c>
       <c r="N64" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE101</t>
-        </is>
-      </c>
-      <c r="O64" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O64" s="4" t="inlineStr">
+        <is>
+          <t>PO-0033</t>
+        </is>
+      </c>
       <c r="P64" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -35112,13 +35140,17 @@
       </c>
       <c r="N69" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE108</t>
-        </is>
-      </c>
-      <c r="O69" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O69" s="4" t="inlineStr">
+        <is>
+          <t>PO-0034</t>
+        </is>
+      </c>
       <c r="P69" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix BOM SKU aggregation, SO grid onclick, Check Material buttons, layout and spacing improvements
- Aggregate BOM rows by SKU_ID at load time so Hot Metal/billets etc. show as single consolidated cards
- Tree node counts now reflect aggregated (unique SKU) count not raw row count
- Remove onclick from SO grid rows — material panel opens only via Check Material button
- Rename Mat buttons to Check Material with cube icon in both SO and PO tables
- Fix template literal syntax error in SO grid row that was breaking all tab navigation
- Two-column layout for BOM detail hero: text left, metrics 2x2 grid right
- Balance KPI strip top/bottom padding; increase card row-gap and padding

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APS_BF_SMS_RM.xlsx
+++ b/APS_BF_SMS_RM.xlsx
@@ -8549,7 +8549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" customWidth="1" style="35" min="1" max="4"/>
@@ -8933,6 +8933,23 @@
       <c r="D19" t="inlineStr">
         <is>
           <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>REQ-1776050729715</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>FG-WR-SAE1008-80</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
         </is>
       </c>
     </row>
@@ -30867,7 +30884,7 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>PO-0025</t>
+          <t>PO-0004</t>
         </is>
       </c>
       <c r="P4" s="4" t="inlineStr">
@@ -30933,7 +30950,7 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>PO-0034</t>
+          <t>PO-0005</t>
         </is>
       </c>
       <c r="P5" s="4" t="inlineStr">
@@ -30999,7 +31016,7 @@
       </c>
       <c r="O6" s="10" t="inlineStr">
         <is>
-          <t>PO-0021</t>
+          <t>PO-0002</t>
         </is>
       </c>
       <c r="P6" s="10" t="inlineStr">
@@ -31065,7 +31082,7 @@
       </c>
       <c r="O7" s="11" t="inlineStr">
         <is>
-          <t>PO-0007</t>
+          <t>PO-0001</t>
         </is>
       </c>
       <c r="P7" s="11" t="inlineStr">
@@ -31131,7 +31148,7 @@
       </c>
       <c r="O8" s="10" t="inlineStr">
         <is>
-          <t>PO-0017</t>
+          <t>PO-0003</t>
         </is>
       </c>
       <c r="P8" s="10" t="inlineStr">
@@ -31197,7 +31214,7 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>PO-0027</t>
+          <t>PO-0030</t>
         </is>
       </c>
       <c r="P9" s="4" t="inlineStr">
@@ -31263,7 +31280,7 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>PO-0038</t>
+          <t>PO-0039</t>
         </is>
       </c>
       <c r="P10" s="4" t="inlineStr">
@@ -31527,7 +31544,7 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>PO-0030</t>
+          <t>PO-0031</t>
         </is>
       </c>
       <c r="P14" s="4" t="inlineStr">
@@ -31659,7 +31676,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>PO-0038</t>
+          <t>PO-0039</t>
         </is>
       </c>
       <c r="P16" s="4" t="inlineStr">
@@ -31857,7 +31874,7 @@
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>PO-0037</t>
+          <t>PO-0038</t>
         </is>
       </c>
       <c r="P19" s="4" t="inlineStr">
@@ -31989,7 +32006,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>PO-0032</t>
+          <t>PO-0033</t>
         </is>
       </c>
       <c r="P21" s="4" t="inlineStr">
@@ -32055,7 +32072,7 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>PO-0030</t>
+          <t>PO-0031</t>
         </is>
       </c>
       <c r="P22" s="4" t="inlineStr">
@@ -32253,7 +32270,7 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>PO-0031</t>
+          <t>PO-0032</t>
         </is>
       </c>
       <c r="P25" s="4" t="inlineStr">
@@ -32583,7 +32600,7 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>PO-0033</t>
+          <t>PO-0034</t>
         </is>
       </c>
       <c r="P30" s="4" t="inlineStr">
@@ -33573,7 +33590,7 @@
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>PO-0027</t>
+          <t>PO-0030</t>
         </is>
       </c>
       <c r="P45" s="4" t="inlineStr">
@@ -33705,7 +33722,7 @@
       </c>
       <c r="O47" s="4" t="inlineStr">
         <is>
-          <t>PO-0036</t>
+          <t>PO-0037</t>
         </is>
       </c>
       <c r="P47" s="4" t="inlineStr">
@@ -33771,7 +33788,7 @@
       </c>
       <c r="O48" s="4" t="inlineStr">
         <is>
-          <t>PO-0036</t>
+          <t>PO-0037</t>
         </is>
       </c>
       <c r="P48" s="4" t="inlineStr">
@@ -34624,13 +34641,17 @@
       </c>
       <c r="N61" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE100</t>
-        </is>
-      </c>
-      <c r="O61" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O61" s="4" t="inlineStr">
+        <is>
+          <t>PO-0041</t>
+        </is>
+      </c>
       <c r="P61" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -34691,7 +34712,7 @@
       </c>
       <c r="O62" s="4" t="inlineStr">
         <is>
-          <t>PO-0035</t>
+          <t>PO-0036</t>
         </is>
       </c>
       <c r="P62" s="4" t="inlineStr">
@@ -34823,7 +34844,7 @@
       </c>
       <c r="O64" s="4" t="inlineStr">
         <is>
-          <t>PO-0033</t>
+          <t>PO-0034</t>
         </is>
       </c>
       <c r="P64" s="4" t="inlineStr">
@@ -35016,13 +35037,17 @@
       </c>
       <c r="N67" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE104</t>
-        </is>
-      </c>
-      <c r="O67" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O67" s="4" t="inlineStr">
+        <is>
+          <t>PO-0042</t>
+        </is>
+      </c>
       <c r="P67" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -35078,13 +35103,17 @@
       </c>
       <c r="N68" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE106</t>
-        </is>
-      </c>
-      <c r="O68" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O68" s="4" t="inlineStr">
+        <is>
+          <t>PO-0039</t>
+        </is>
+      </c>
       <c r="P68" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -35145,7 +35174,7 @@
       </c>
       <c r="O69" s="4" t="inlineStr">
         <is>
-          <t>PO-0034</t>
+          <t>PO-0035</t>
         </is>
       </c>
       <c r="P69" s="4" t="inlineStr">
@@ -35206,13 +35235,17 @@
       </c>
       <c r="N70" s="4" t="inlineStr">
         <is>
-          <t>CMP-CHQ100</t>
-        </is>
-      </c>
-      <c r="O70" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O70" s="4" t="inlineStr">
+        <is>
+          <t>PO-0040</t>
+        </is>
+      </c>
       <c r="P70" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -35268,13 +35301,17 @@
       </c>
       <c r="N71" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE100</t>
-        </is>
-      </c>
-      <c r="O71" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O71" s="4" t="inlineStr">
+        <is>
+          <t>PO-0001</t>
+        </is>
+      </c>
       <c r="P71" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -35330,13 +35367,17 @@
       </c>
       <c r="N72" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE100</t>
-        </is>
-      </c>
-      <c r="O72" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O72" s="4" t="inlineStr">
+        <is>
+          <t>PO-0005</t>
+        </is>
+      </c>
       <c r="P72" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -35392,13 +35433,17 @@
       </c>
       <c r="N73" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE101</t>
-        </is>
-      </c>
-      <c r="O73" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O73" s="4" t="inlineStr">
+        <is>
+          <t>PO-0006</t>
+        </is>
+      </c>
       <c r="P73" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -35454,13 +35499,17 @@
       </c>
       <c r="N74" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE101</t>
-        </is>
-      </c>
-      <c r="O74" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O74" s="4" t="inlineStr">
+        <is>
+          <t>PO-0002</t>
+        </is>
+      </c>
       <c r="P74" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -35516,13 +35565,17 @@
       </c>
       <c r="N75" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE103</t>
-        </is>
-      </c>
-      <c r="O75" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O75" s="4" t="inlineStr">
+        <is>
+          <t>PO-0007</t>
+        </is>
+      </c>
       <c r="P75" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -35578,13 +35631,17 @@
       </c>
       <c r="N76" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE103</t>
-        </is>
-      </c>
-      <c r="O76" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O76" s="4" t="inlineStr">
+        <is>
+          <t>PO-0003</t>
+        </is>
+      </c>
       <c r="P76" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -35640,13 +35697,17 @@
       </c>
       <c r="N77" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE104</t>
-        </is>
-      </c>
-      <c r="O77" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O77" s="4" t="inlineStr">
+        <is>
+          <t>PO-0010</t>
+        </is>
+      </c>
       <c r="P77" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -35702,13 +35763,17 @@
       </c>
       <c r="N78" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE106</t>
-        </is>
-      </c>
-      <c r="O78" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O78" s="4" t="inlineStr">
+        <is>
+          <t>PO-0008</t>
+        </is>
+      </c>
       <c r="P78" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -35764,13 +35829,17 @@
       </c>
       <c r="N79" s="4" t="inlineStr">
         <is>
-          <t>CMP-SAE108</t>
-        </is>
-      </c>
-      <c r="O79" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O79" s="4" t="inlineStr">
+        <is>
+          <t>PO-0009</t>
+        </is>
+      </c>
       <c r="P79" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -35826,13 +35895,17 @@
       </c>
       <c r="N80" s="4" t="inlineStr">
         <is>
-          <t>CMP-CHQ100</t>
-        </is>
-      </c>
-      <c r="O80" s="4" t="n"/>
+          <t>APS_RELEASED</t>
+        </is>
+      </c>
+      <c r="O80" s="4" t="inlineStr">
+        <is>
+          <t>PO-0004</t>
+        </is>
+      </c>
       <c r="P80" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>

</xml_diff>